<commit_message>
fix(ui): canlı önizleme ve puan boyutu ayarı eklendi
</commit_message>
<xml_diff>
--- a/static/NotGiris/TAPU303_Final.xlsx
+++ b/static/NotGiris/TAPU303_Final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erdem/.gemini/antigravity/scratch/sinav-kagidi/static/NotGiris/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{106B244E-6FD5-A64F-862B-96BC0221CBC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{371C1CC7-CE9A-2249-8675-B46ADB5822BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="680" windowWidth="17280" windowHeight="20240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4360" yWindow="680" windowWidth="30200" windowHeight="20260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Page 1" sheetId="1" r:id="rId1"/>
@@ -775,13 +775,13 @@
       <sz val="8"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1136,8 +1136,10 @@
     <col min="2" max="2" width="25.5" customWidth="1"/>
     <col min="3" max="3" width="20.33203125" customWidth="1"/>
     <col min="4" max="4" width="20.5" customWidth="1"/>
-    <col min="5" max="5" width="20.33203125" customWidth="1"/>
-    <col min="6" max="8" width="25.5" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -1252,7 +1254,7 @@
         <v>18</v>
       </c>
       <c r="G5" s="3">
-        <v>48</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -1321,7 +1323,7 @@
         <v>38</v>
       </c>
       <c r="G8" s="3">
-        <v>36</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -1367,7 +1369,7 @@
         <v>47</v>
       </c>
       <c r="G10" s="3">
-        <v>55</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -1390,7 +1392,7 @@
         <v>18</v>
       </c>
       <c r="G11" s="3">
-        <v>65</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="13.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1482,7 +1484,7 @@
         <v>68</v>
       </c>
       <c r="G15" s="3">
-        <v>55</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -1505,7 +1507,7 @@
         <v>33</v>
       </c>
       <c r="G16" s="3">
-        <v>30</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -1597,7 +1599,7 @@
         <v>38</v>
       </c>
       <c r="G20" s="3">
-        <v>23</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1643,7 +1645,7 @@
         <v>68</v>
       </c>
       <c r="G22" s="3">
-        <v>50</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -1666,7 +1668,7 @@
         <v>33</v>
       </c>
       <c r="G23" s="3">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1735,7 +1737,7 @@
         <v>38</v>
       </c>
       <c r="G26" s="3">
-        <v>43</v>
+        <v>73</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1804,7 +1806,7 @@
         <v>18</v>
       </c>
       <c r="G29" s="3">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -1850,7 +1852,7 @@
         <v>18</v>
       </c>
       <c r="G31" s="3">
-        <v>40</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -1873,7 +1875,7 @@
         <v>38</v>
       </c>
       <c r="G32" s="3">
-        <v>53</v>
+        <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -1896,7 +1898,7 @@
         <v>68</v>
       </c>
       <c r="G33" s="3">
-        <v>48</v>
+        <v>78</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1919,7 +1921,7 @@
         <v>38</v>
       </c>
       <c r="G34" s="3">
-        <v>46</v>
+        <v>70</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -1965,7 +1967,7 @@
         <v>18</v>
       </c>
       <c r="G36" s="3">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1988,7 +1990,7 @@
         <v>18</v>
       </c>
       <c r="G37" s="3">
-        <v>35</v>
+        <v>55</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2034,7 +2036,7 @@
         <v>68</v>
       </c>
       <c r="G39" s="3">
-        <v>45</v>
+        <v>75</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -2057,7 +2059,7 @@
         <v>18</v>
       </c>
       <c r="G40" s="3">
-        <v>40</v>
+        <v>50</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2080,7 +2082,7 @@
         <v>68</v>
       </c>
       <c r="G41" s="3">
-        <v>55</v>
+        <v>75</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2103,7 +2105,7 @@
         <v>38</v>
       </c>
       <c r="G42" s="3">
-        <v>50</v>
+        <v>70</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -2126,7 +2128,7 @@
         <v>18</v>
       </c>
       <c r="G43" s="3">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2172,7 +2174,7 @@
         <v>38</v>
       </c>
       <c r="G45" s="3">
-        <v>61</v>
+        <v>71</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2218,7 +2220,7 @@
         <v>38</v>
       </c>
       <c r="G47" s="3">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2241,7 +2243,7 @@
         <v>38</v>
       </c>
       <c r="G48" s="3">
-        <v>53</v>
+        <v>73</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2333,7 +2335,7 @@
         <v>68</v>
       </c>
       <c r="G52" s="3">
-        <v>65</v>
+        <v>75</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -2356,7 +2358,7 @@
         <v>33</v>
       </c>
       <c r="G53" s="3">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2379,7 +2381,7 @@
         <v>68</v>
       </c>
       <c r="G54" s="3">
-        <v>56</v>
+        <v>76</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2448,7 +2450,7 @@
         <v>38</v>
       </c>
       <c r="G57" s="3">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2471,7 +2473,7 @@
         <v>18</v>
       </c>
       <c r="G58" s="3">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2540,7 +2542,7 @@
         <v>68</v>
       </c>
       <c r="G61" s="3">
-        <v>60</v>
+        <v>75</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2563,7 +2565,7 @@
         <v>38</v>
       </c>
       <c r="G62" s="3">
-        <v>45</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>